<commit_message>
syllabus links and manual slot editing
</commit_message>
<xml_diff>
--- a/src/test.xlsx
+++ b/src/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rjooske/akiko/akiko-blastoise/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{486379C2-D244-F140-8D64-517394B0E5F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9F11FC-73F0-CB4C-89EF-32D212664095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="開設科目一覧" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">開設科目一覧!$A$1:$K$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">開設科目一覧!$A$1:$K$13</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="66">
   <si>
     <t>開設母体</t>
   </si>
@@ -210,6 +210,24 @@
   </si>
   <si>
     <t>123abc</t>
+  </si>
+  <si>
+    <t>AA00008</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>5.0</t>
+  </si>
+  <si>
+    <t>3-4</t>
+  </si>
+  <si>
+    <t>秋C</t>
+  </si>
+  <si>
+    <t>NT3,4</t>
   </si>
 </sst>
 </file>
@@ -922,7 +940,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
@@ -1051,23 +1069,23 @@
     </row>
     <row r="7" spans="1:19" ht="24">
       <c r="A7" s="20" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C7" s="22"/>
       <c r="D7" s="22" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="H7" s="22"/>
       <c r="I7" s="21"/>
@@ -1082,25 +1100,25 @@
       <c r="R7" s="21"/>
       <c r="S7" s="26"/>
     </row>
-    <row r="8" spans="1:19" ht="36">
+    <row r="8" spans="1:19" ht="24">
       <c r="A8" s="20" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C8" s="22"/>
       <c r="D8" s="22" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="H8" s="22"/>
       <c r="I8" s="21"/>
@@ -1115,25 +1133,25 @@
       <c r="R8" s="21"/>
       <c r="S8" s="26"/>
     </row>
-    <row r="9" spans="1:19" ht="24">
+    <row r="9" spans="1:19" ht="36">
       <c r="A9" s="20" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C9" s="22"/>
       <c r="D9" s="22" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>35</v>
+        <v>52</v>
+      </c>
+      <c r="G9" s="27" t="s">
+        <v>53</v>
       </c>
       <c r="H9" s="22"/>
       <c r="I9" s="21"/>
@@ -1148,25 +1166,25 @@
       <c r="R9" s="21"/>
       <c r="S9" s="26"/>
     </row>
-    <row r="10" spans="1:19" ht="48">
+    <row r="10" spans="1:19" ht="24">
       <c r="A10" s="20" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="22" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="H10" s="22"/>
       <c r="I10" s="21"/>
@@ -1181,25 +1199,25 @@
       <c r="R10" s="21"/>
       <c r="S10" s="26"/>
     </row>
-    <row r="11" spans="1:19" ht="24">
+    <row r="11" spans="1:19" ht="48">
       <c r="A11" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C11" s="22"/>
       <c r="D11" s="22" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H11" s="22"/>
       <c r="I11" s="21"/>
@@ -1215,39 +1233,72 @@
       <c r="S11" s="26"/>
     </row>
     <row r="12" spans="1:19" ht="24">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" s="22"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="25"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="25"/>
+      <c r="O12" s="23"/>
+      <c r="P12" s="20"/>
+      <c r="Q12" s="21"/>
+      <c r="R12" s="21"/>
+      <c r="S12" s="26"/>
+    </row>
+    <row r="13" spans="1:19" ht="24">
+      <c r="A13" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6" t="s">
+      <c r="C13" s="6"/>
+      <c r="D13" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H13" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="16"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="10"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="16"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.45500000000000002" bottom="0.55000000000000004" header="0.3" footer="0.3"/>

</xml_diff>